<commit_message>
inserting records into tables
</commit_message>
<xml_diff>
--- a/Pham_Ex3A_tables.xlsx
+++ b/Pham_Ex3A_tables.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Longley\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Longley\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{914C41BC-3EC9-406A-BA4A-CB4344CEF143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB84E878-1E77-4D5F-9F68-945ED34E1967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="10500" windowWidth="19200" windowHeight="10500" xr2:uid="{21EA6C4E-3D97-4843-80D7-8EA301420543}"/>
+    <workbookView xWindow="2325" yWindow="5310" windowWidth="14250" windowHeight="9750" xr2:uid="{21EA6C4E-3D97-4843-80D7-8EA301420543}"/>
   </bookViews>
   <sheets>
     <sheet name="customers" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
   <si>
     <t>customer_id</t>
   </si>
@@ -106,6 +106,30 @@
   </si>
   <si>
     <t>tip_amount</t>
+  </si>
+  <si>
+    <t>James Sera</t>
+  </si>
+  <si>
+    <t>111 S Michigan Avenue, Chicago, IL 60603</t>
+  </si>
+  <si>
+    <t>Buddy</t>
+  </si>
+  <si>
+    <t>Golden Retriever</t>
+  </si>
+  <si>
+    <t>Liam Carter</t>
+  </si>
+  <si>
+    <t>completed</t>
+  </si>
+  <si>
+    <t>Good behavior</t>
+  </si>
+  <si>
+    <t>card</t>
   </si>
 </sst>
 </file>
@@ -153,10 +177,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -491,8 +517,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1F9F637-C64A-456D-B205-D19CFDB6BC41}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -511,6 +540,23 @@
         <v>4</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2">
+        <v>5056272144</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2">
+        <v>3.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -518,7 +564,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{302C1B71-80D6-4F9C-AFCC-470E071F2BDF}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -538,6 +584,23 @@
         <v>8</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2">
+        <v>4.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -545,8 +608,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0861F399-154E-47FB-A569-F1C6C8BE09D1}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -562,6 +628,20 @@
         <v>10</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2">
+        <v>3126001001</v>
+      </c>
+      <c r="D2">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -569,7 +649,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB9DE657-4053-4802-A43F-7CEA2545AA9C}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -598,6 +678,32 @@
         <v>16</v>
       </c>
     </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3">
+        <v>46113</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F2" s="4">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -605,7 +711,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9775E87-8EA7-4780-8DE9-C4A7B5109313}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -628,6 +734,26 @@
         <v>21</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="3">
+        <v>46113</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>